<commit_message>
update 20 defects of requirement 2
</commit_message>
<xml_diff>
--- a/spreadsheet/test_cases_checklist.xlsx
+++ b/spreadsheet/test_cases_checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Workspace\HCMUS\Test\Week 1\HW1\spreadsheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6919329B-D87D-4BEC-90E8-E315E2ADCCB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EA890B6-07E6-41DE-918C-DA6904AEECF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="110">
   <si>
     <t>No.</t>
   </si>
@@ -55,6 +55,9 @@
     <t>Actual Result</t>
   </si>
   <si>
+    <t>AI Generated</t>
+  </si>
+  <si>
     <t>TC01</t>
   </si>
   <si>
@@ -67,49 +70,313 @@
     <t>v1.0</t>
   </si>
   <si>
+    <t>Kiểm tra tính năng Bật/Tắt (Power On/Off) của quạt bằng nút bấm vật lý trên thân quạt.</t>
+  </si>
+  <si>
+    <t>Quạt đứng Asiavina D16022-DV0 đã được cắm vào nguồn điện xoay chiều 220V ổn định. Tất cả các nút bấm tốc độ (1, 2, 3) đang ở trạng thái nảy lên (tắt).</t>
+  </si>
+  <si>
+    <t>1. Nhấn nút tốc độ 1 trên bảng điều khiển cơ.
+2. Quan sát hoạt động của cánh quạt.
+3. Nhấn nút "OFF" (nút nguồn/tắt) trên bảng điều khiển.</t>
+  </si>
+  <si>
+    <t>Nút nhấn vật lý: nút 1 và nút OFF</t>
+  </si>
+  <si>
+    <t>1. Khi nhấn nút 1, quạt khởi động, cánh quạt quay ở tốc độ nhẹ, ổn định.
+2. Khi nhấn nút OFF, quạt ngừng cấp điện, cánh quạt quay chậm dần rồi dừng hẳn.</t>
+  </si>
+  <si>
+    <t>Yes (Reviewed)</t>
+  </si>
+  <si>
     <t>TC02</t>
   </si>
   <si>
+    <t>Kiểm tra chức năng thay đổi tốc độ gió (Speed Control) từ mức 1 đến mức 3.</t>
+  </si>
+  <si>
+    <t>Quạt đang chạy ở tốc độ 1.</t>
+  </si>
+  <si>
+    <t>1. Nhấn phím số 2 trên bảng điều khiển.
+2. Nhấn phím số 3 trên bảng điều khiển.</t>
+  </si>
+  <si>
+    <t>Nút nhấn vật lý: nút 2 và nút 3</t>
+  </si>
+  <si>
+    <t>1. Khi nhấn phím 2, phím 1 tự nảy lên, phím 2 giữ nguyên ở trạng thái nhấn, tốc độ quạt tăng lên rõ rệt (mức trung bình).
+2. Khi nhấn phím 3, phím 2 tự nảy lên, phím 3 giữ nguyên ở trạng thái nhấn, tốc độ quạt tăng lên mức tối đa.</t>
+  </si>
+  <si>
     <t>TC03</t>
   </si>
   <si>
+    <t>Kiểm tra tính năng xoay tu năng (Oscillation) kết hợp tốc độ gió mức 3. (Phát hiện lỗi tiếng kêu động cơ).</t>
+  </si>
+  <si>
+    <t>Quạt đã được bật ở tốc độ 3.</t>
+  </si>
+  <si>
+    <t>1. Nhấn chốt giật tu năng cơ học trên hộp số động cơ xuống để kích hoạt chế độ xoay.
+2. Để quạt chạy liên tục trong 5 phút.
+3. Nhấc chốt giật tu năng lên để tắt chế độ xoay.</t>
+  </si>
+  <si>
+    <t>Chốt giật tu năng cơ học, phím tốc độ 3</t>
+  </si>
+  <si>
+    <t>1. Quạt xoay ngang đều từ trái qua phải và ngược lại với góc quay khoảng 90 độ.
+2. Không phát ra tiếng kêu lạ từ ổ trục hay động cơ.
+3. Khi nhấc chốt giật lên, quạt dừng xoay ở hướng hiện tại và tiếp tục thổi gió cố định.</t>
+  </si>
+  <si>
     <t>TC04</t>
   </si>
   <si>
+    <t>Kiểm tra độ nhạy và cơ chế phản hồi cơ học của phím bấm điều khiển. (Phát hiện lỗi kẹt phím).</t>
+  </si>
+  <si>
+    <t>Quạt đang ở trạng thái OFF.</t>
+  </si>
+  <si>
+    <t>1. Nhấn phím số 2 xuống.
+2. Nhấn phím số 3 xuống liên tục nhiều lần (khoảng 30 lần) để kiểm tra cơ cấu lò xo cơ học.
+3. Quan sát xem phím 2 có tự động nảy lên mỗi khi phím 3 được nhấn hay không.</t>
+  </si>
+  <si>
+    <t>Nhấn liên tục các phím cơ 2 và 3</t>
+  </si>
+  <si>
+    <t>Mỗi lần nhấn một phím tốc độ khác, phím đang nhấn trước đó phải tự động giải phóng (nảy lên) hoàn toàn mà không bị kẹt.</t>
+  </si>
+  <si>
     <t>TC05</t>
   </si>
   <si>
+    <t>Reliability</t>
+  </si>
+  <si>
+    <t>Kiểm tra tính năng xoay tu năng cơ liên tục (Oscillation Wear Test). (Phát hiện lỗi tu năng cơ).</t>
+  </si>
+  <si>
+    <t>Quạt đặt trên mặt phẳng, bật tốc độ 2.</t>
+  </si>
+  <si>
+    <t>1. Nhấn chốt tu năng xuống để quạt xoay.
+2. Cho quạt chạy liên tục trong 15 phút.
+3. Quan sát hoạt động cơ học ở các góc biên trái và phải.</t>
+  </si>
+  <si>
+    <t>Chạy liên tục tốc độ 2 kết hợp xoay tu năng</t>
+  </si>
+  <si>
+    <t>Quạt xoay đảo chiều mượt mà ở các góc biên, không bị khựng lại hay phát ra tiếng kêu từ bánh răng truyền động.</t>
+  </si>
+  <si>
     <t>TC06</t>
   </si>
   <si>
+    <t>Kiểm tra độ ổn định của ren siết khóa chiều cao thân quạt dưới tác động của lực rung cơ học. (Phát hiện lỗi ren siết).</t>
+  </si>
+  <si>
+    <t>Điều chỉnh quạt đứng ở độ cao tối đa (1.2m), siết chặt vòng cổ ren khóa chiều cao bằng tay.</t>
+  </si>
+  <si>
+    <t>1. Bật quạt chạy ở tốc độ lớn nhất (mức 3).
+2. Nhấn tu năng cho quạt xoay liên tục trong 10 phút.
+3. Kiểm tra xem chiều cao thân quạt có bị thay đổi không.</t>
+  </si>
+  <si>
+    <t>Quạt kéo cao tối đa 1.2m, chạy tốc độ 3 xoay tu năng</t>
+  </si>
+  <si>
+    <t>Vòng khóa giữ nguyên vị trí, quạt đứng vững ở độ cao 1.2m, không bị sụt độ cao dưới tác động của lực rung động cơ.</t>
+  </si>
+  <si>
     <t>TC07</t>
   </si>
   <si>
+    <t>Safety</t>
+  </si>
+  <si>
+    <t>Kiểm tra khả năng hoạt động liên tục ở tải cao và cơ cấu bảo vệ quá nhiệt (Thermal Cutoff). (Phát hiện lỗi cầu chì nhiệt).</t>
+  </si>
+  <si>
+    <t>Đặt quạt trong phòng kín nhỏ có nhiệt độ không khí cao (~36°C).</t>
+  </si>
+  <si>
+    <t>1. Bật quạt chạy ở tốc độ 3 liên tục trong 4 tiếng.
+2. Theo dõi nhiệt độ vỏ động cơ và trạng thái quay của quạt.</t>
+  </si>
+  <si>
+    <t>Chạy liên tục tốc độ 3, nhiệt độ phòng ~36°C trong 4 tiếng</t>
+  </si>
+  <si>
+    <t>Động cơ nóng lên trong giới hạn cho phép (&lt;75°C), quạt chạy liên tục ổn định. Nếu quá nhiệt cực hạn, cầu chì nhiệt phải ngắt nguồn bảo vệ chống cháy nổ.</t>
+  </si>
+  <si>
     <t>TC08</t>
   </si>
   <si>
+    <t>Stability</t>
+  </si>
+  <si>
+    <t>Kiểm tra độ vững chãi của đế quạt khi hoạt động ở tốc độ tối đa.</t>
+  </si>
+  <si>
+    <t>Quạt đặt trên mặt sàn gạch phẳng, khô ráo.</t>
+  </si>
+  <si>
+    <t>1. Bật quạt chạy ở tốc độ 3.
+2. Quan sát độ rung lắc của thân và đế quạt trong 5 phút.</t>
+  </si>
+  <si>
+    <t>Chạy tốc độ 3 cố định trên sàn phẳng</t>
+  </si>
+  <si>
+    <t>Thân quạt đứng vững, đế quạt bám chắc mặt sàn, độ rung lắc nằm trong biên độ nhỏ cho phép (&lt;5mm tại đỉnh lồng quạt).</t>
+  </si>
+  <si>
     <t>TC09</t>
   </si>
   <si>
+    <t>Physical Edge Case</t>
+  </si>
+  <si>
+    <t>Kiểm tra độ vững chãi và hiện tượng dịch chuyển cơ học (walk/drift) trên mặt sàn trơn trượt có góc dốc nhẹ. (Edge Case 1)</t>
+  </si>
+  <si>
+    <t>Đặt quạt trên mặt sàn gạch men dốc nghiêng 2 độ và có phủ một lớp nước mỏng (trơn trượt).</t>
+  </si>
+  <si>
+    <t>1. Bật quạt chạy ở tốc độ cao nhất (Tốc độ 3).
+2. Nhấn chốt tu năng cho quạt xoay 90 độ liên tục.
+3. Quan sát xem đế quạt có bị dịch chuyển vị trí cơ học hay không sau 5 phút.</t>
+  </si>
+  <si>
+    <t>Sàn gạch men dốc 2 độ dính nước, chạy tốc độ 3 xoay tu năng</t>
+  </si>
+  <si>
+    <t>Đế quạt (nhờ đệm cao su) vẫn bám chắc vào mặt sàn, quạt đứng yên tại vị trí ban đầu, không bị trượt hay tự dịch chuyển cơ học dưới tác động của lực ly tâm và mô-men quay.</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
     <t>TC10</t>
   </si>
   <si>
+    <t>Kiểm tra ảnh hưởng cơ học của việc đi dây nguồn khi quạt thực hiện chuyển động xoay tu năng ở góc tối đa. (Edge Case 2)</t>
+  </si>
+  <si>
+    <t>Dây nguồn của quạt được cắm vào ổ điện trên tường sao cho độ căng của dây vừa đủ thẳng khi quạt hướng chính diện.</t>
+  </si>
+  <si>
+    <t>1. Bật quạt chạy ở tốc độ 2.
+2. Nhấn chốt tu năng cho quạt xoay.
+3. Quan sát trạng thái cơ học của dây nguồn và phích cắm khi quạt xoay sang biên trái góc 45 độ (góc tối đa).</t>
+  </si>
+  <si>
+    <t>Cắm dây nguồn căng vừa đủ thẳng, bật xoay tu năng</t>
+  </si>
+  <si>
+    <t>Dây nguồn phải có đủ độ chùng dự phòng. Khi đầu quạt xoay đến các góc biên, phích cắm không bị kéo căng, chân phích cắm bám chặt trong ổ cắm điện ổn định.</t>
+  </si>
+  <si>
     <t>TC11</t>
   </si>
   <si>
+    <t>Kiểm tra phản ứng cơ-nhiệt của động cơ và tu năng khi quạt đứng bị nghiêng góc nhẹ. (Edge Case 3)</t>
+  </si>
+  <si>
+    <t>Đặt quạt trên mặt sàn thảm mềm làm thân quạt bị nghiêng nhẹ góc 5 độ sang một bên.</t>
+  </si>
+  <si>
+    <t>1. Bật quạt chạy ở tốc độ 2.
+2. Nhấn chốt tu năng cho quạt xoay ngang liên tục trong 10 phút.
+3. Theo dõi cơ cấu tu năng xoay và nhiệt độ hộp số.</t>
+  </si>
+  <si>
+    <t>Đặt quạt trên thảm nghiêng 5 độ, chạy tốc độ 2 xoay tu năng</t>
+  </si>
+  <si>
+    <t>Cơ cấu trục quay khớp cổ và tu năng hoạt động bình thường dưới tải trọng nghiêng, góc xoay không bị cản trở, động cơ không bị quá tải nhiệt.</t>
+  </si>
+  <si>
     <t>TC12</t>
   </si>
   <si>
+    <t>Kiểm tra hoạt động bật/tắt của cơ cấu túp năng khi thay đổi trạng thái giật/nhả liên tục.</t>
+  </si>
+  <si>
+    <t>1. Nhấn chốt giật tu năng xuống, đợi quạt quay góc 45 độ, sau đó kéo chốt giật lên.
+2. Thực hiện lặp lại thao tác này 10 lần liên tục.</t>
+  </si>
+  <si>
+    <t>Giật/nhả chốt tu năng cơ 10 lần liên tục</t>
+  </si>
+  <si>
+    <t>Cơ cấu tu năng cơ học hoạt động nhạy, bắt khớp và nhả khớp bánh răng mượt mà, không bị kẹt hay trượt răng khi đổi trạng thái đột ngột.</t>
+  </si>
+  <si>
     <t>TC13</t>
   </si>
   <si>
+    <t>Kiểm tra tính chắc chắn và an toàn của lồng quạt bảo vệ dưới lực tác động vật lý bên ngoài.</t>
+  </si>
+  <si>
+    <t>Quạt đã được tắt điện.</t>
+  </si>
+  <si>
+    <t>1. Dùng tay ấn lực nhẹ (~20N) lên các nan lồng quạt phía trước và phía sau.
+2. Kiểm tra xem nan lồng quạt có bị biến dạng chạm vào cánh quạt bên trong hay không.</t>
+  </si>
+  <si>
+    <t>Tác dụng lực ấn 20N lên nan lồng quạt</t>
+  </si>
+  <si>
+    <t>Lồng quạt kim loại chắc chắn, không bị biến dạng dễ dàng, khoảng cách an toàn giữa lồng quạt và cánh quạt được duy trì tốt (khoảng cách &gt;1.5cm).</t>
+  </si>
+  <si>
     <t>TC14</t>
   </si>
   <si>
+    <t>Kiểm tra tính năng khóa/mở khớp xoay đứng (điều chỉnh góc ngẩng/cúi đầu quạt).</t>
+  </si>
+  <si>
+    <t>1. Dùng tay điều chỉnh đầu quạt ngửa lên góc tối đa (khoảng 30 độ), sau đó gập xuống góc tối đa (khoảng 15 độ).
+2. Bật quạt chạy ở tốc độ 3 và kiểm tra xem đầu quạt có giữ nguyên góc nghiêng hay tự động gục xuống.</t>
+  </si>
+  <si>
+    <t>Góc cúi/ngẩng cơ học của đầu quạt</t>
+  </si>
+  <si>
+    <t>Khớp cổ quạt di chuyển nấc cơ học chắc chắn. Khi quạt chạy tốc độ 3, đầu quạt giữ nguyên góc điều chỉnh mà không bị xê dịch tự do dưới lực đẩy của gió.</t>
+  </si>
+  <si>
     <t>TC15</t>
   </si>
   <si>
-    <t>AI Generated</t>
+    <t>Performance</t>
+  </si>
+  <si>
+    <t>Kiểm tra độ ồn của động cơ ở khoảng cách 1m tại các tốc độ hoạt động khác nhau.</t>
+  </si>
+  <si>
+    <t>Đặt quạt trong phòng ngủ có độ ồn môi trường thấp (&lt;30dB).</t>
+  </si>
+  <si>
+    <t>1. Bật quạt ở tốc độ 1, dùng máy đo độ ồn đặt cách quạt 1m đo độ ồn.
+2. Lặp lại với tốc độ 2 và tốc độ 3.</t>
+  </si>
+  <si>
+    <t>Đo độ ồn ở tốc độ 1, 2, 3 cách quạt 1m</t>
+  </si>
+  <si>
+    <t>Độ ồn ở mức 1 phải đạt chuẩn Silent/Sleep (&lt;38dB), mức 2 &lt;45dB và mức 3 &lt;52dB.</t>
   </si>
 </sst>
 </file>
@@ -510,20 +777,22 @@
   <dimension ref="A1:L16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="6" customWidth="1"/>
-    <col min="2" max="2" width="13" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="30" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="35" customWidth="1"/>
+    <col min="1" max="1" width="4.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="34.90625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="25" customWidth="1"/>
-    <col min="8" max="8" width="40" customWidth="1"/>
-    <col min="9" max="9" width="20" customWidth="1"/>
-    <col min="10" max="11" width="35" customWidth="1"/>
-    <col min="12" max="12" width="14" customWidth="1"/>
+    <col min="8" max="8" width="39.90625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="34.90625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -558,368 +827,548 @@
         <v>10</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="96" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
+        <v>15</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>20</v>
+      </c>
       <c r="K2" s="3"/>
-      <c r="L2" s="2"/>
-    </row>
-    <row r="3" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L2" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="96" x14ac:dyDescent="0.35">
       <c r="A3" s="4">
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="5"/>
+        <v>15</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>27</v>
+      </c>
       <c r="K3" s="5"/>
-      <c r="L3" s="4"/>
-    </row>
-    <row r="4" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L3" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="112" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
+        <v>15</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>33</v>
+      </c>
       <c r="K4" s="3"/>
-      <c r="L4" s="2"/>
-    </row>
-    <row r="5" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L4" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="80" x14ac:dyDescent="0.35">
       <c r="A5" s="4">
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
+        <v>15</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>39</v>
+      </c>
       <c r="K5" s="5"/>
-      <c r="L5" s="4"/>
-    </row>
-    <row r="6" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L5" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="64" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
+        <v>15</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>46</v>
+      </c>
       <c r="K6" s="3"/>
-      <c r="L6" s="2"/>
-    </row>
-    <row r="7" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L6" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="80" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
+        <v>15</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>52</v>
+      </c>
       <c r="K7" s="5"/>
-      <c r="L7" s="4"/>
-    </row>
-    <row r="8" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L7" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="64" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>20</v>
+        <v>53</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>12</v>
+        <v>54</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
+        <v>15</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>59</v>
+      </c>
       <c r="K8" s="3"/>
-      <c r="L8" s="2"/>
-    </row>
-    <row r="9" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L8" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="48" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="K9" s="5"/>
+      <c r="L9" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="4"/>
-    </row>
-    <row r="10" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="10" spans="1:12" ht="80" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>22</v>
+        <v>67</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>12</v>
+        <v>68</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
+        <v>15</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="K10" s="3"/>
-      <c r="L10" s="2"/>
-    </row>
-    <row r="11" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L10" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="80" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>23</v>
+        <v>75</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>12</v>
+        <v>68</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
+        <v>15</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>80</v>
+      </c>
       <c r="K11" s="5"/>
-      <c r="L11" s="4"/>
-    </row>
-    <row r="12" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L11" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="80" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>24</v>
+        <v>81</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>12</v>
+        <v>68</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
+        <v>15</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>86</v>
+      </c>
       <c r="K12" s="3"/>
-      <c r="L12" s="2"/>
-    </row>
-    <row r="13" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L12" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="64" x14ac:dyDescent="0.35">
       <c r="A13" s="4">
         <v>12</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>25</v>
+        <v>87</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
+        <v>15</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="J13" s="5" t="s">
+        <v>91</v>
+      </c>
       <c r="K13" s="5"/>
-      <c r="L13" s="4"/>
-    </row>
-    <row r="14" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L13" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="64" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>26</v>
+        <v>92</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>12</v>
+        <v>54</v>
       </c>
       <c r="D14" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="K14" s="3"/>
+      <c r="L14" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="96" x14ac:dyDescent="0.35">
+      <c r="A15" s="4">
+        <v>14</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E14" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="2"/>
-    </row>
-    <row r="15" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="4">
-        <v>14</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>12</v>
-      </c>
       <c r="D15" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
+        <v>15</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="J15" s="5" t="s">
+        <v>102</v>
+      </c>
       <c r="K15" s="5"/>
-      <c r="L15" s="4"/>
-    </row>
-    <row r="16" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L15" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="48" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>28</v>
+        <v>103</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>12</v>
+        <v>104</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
-      <c r="I16" s="3"/>
-      <c r="J16" s="3"/>
+        <v>15</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>109</v>
+      </c>
       <c r="K16" s="3"/>
-      <c r="L16" s="2"/>
+      <c r="L16" s="2" t="s">
+        <v>21</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
update 15 test case and status
</commit_message>
<xml_diff>
--- a/spreadsheet/test_cases_checklist.xlsx
+++ b/spreadsheet/test_cases_checklist.xlsx
@@ -602,10 +602,19 @@
 2. Khi nhấn nút OFF, quạt ngừng cấp điện, cánh quạt quay chậm dần rồi dừng hẳn.</t>
         </is>
       </c>
-      <c r="K2" s="3" t="n"/>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>[PASS] Quạt khởi động và tắt bình thường khi bấm các phím tương ứng.</t>
+        </is>
+      </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Yes (Reviewed)</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -660,10 +669,19 @@
 2. Khi nhấn phím 3, phím 2 tự nảy lên, phím 3 giữ nguyên ở trạng thái nhấn, tốc độ quạt tăng lên mức tối đa.</t>
         </is>
       </c>
-      <c r="K3" s="5" t="n"/>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>[PASS] Thay đổi tốc độ gió phản hồi đúng trạng thái phím cơ học.</t>
+        </is>
+      </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
           <t>Yes (Reviewed)</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -720,10 +738,19 @@
 3. Khi nhấc chốt giật lên, quạt dừng xoay ở hướng hiện tại và tiếp tục thổi gió cố định.</t>
         </is>
       </c>
-      <c r="K4" s="3" t="n"/>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>[PASS] Tu năng xoay ngang mượt mà, không phát ra tiếng động cơ học lạ.</t>
+        </is>
+      </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
           <t>Yes (Reviewed)</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -778,10 +805,19 @@
           <t>Mỗi lần nhấn một phím tốc độ khác, phím đang nhấn trước đó phải tự động giải phóng (nảy lên) hoàn toàn mà không bị kẹt.</t>
         </is>
       </c>
-      <c r="K5" s="5" t="n"/>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>[PASS] Các phím cơ phản hồi nhạy, phím cũ tự nảy lên mượt mà khi nhấn phím mới.</t>
+        </is>
+      </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
           <t>Yes (Reviewed)</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -836,10 +872,19 @@
           <t>Quạt xoay đảo chiều mượt mà ở các góc biên, không bị khựng lại hay phát ra tiếng kêu từ bánh răng truyền động.</t>
         </is>
       </c>
-      <c r="K6" s="3" t="n"/>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>[PASS] Tu năng cơ bắt khớp và đảo chiều mượt mà ở các góc biên.</t>
+        </is>
+      </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
           <t>Yes (Reviewed)</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -894,10 +939,19 @@
           <t>Vòng khóa giữ nguyên vị trí, quạt đứng vững ở độ cao 1.2m, không bị sụt độ cao dưới tác động của lực rung động cơ.</t>
         </is>
       </c>
-      <c r="K7" s="5" t="n"/>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>[FAIL] Kết quả không ổn định. Khi điều chỉnh tăng chiều cao quá mức thì thân quạt bắt đầu rung lắc tương đối mạnh khi hoạt động, có thể dẫn đến ngã đổ quạt.</t>
+        </is>
+      </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
           <t>Yes (Reviewed)</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -951,10 +1005,19 @@
           <t>Động cơ nóng lên trong giới hạn cho phép (&lt;75°C), quạt chạy liên tục ổn định. Nếu quá nhiệt cực hạn, cầu chì nhiệt phải ngắt nguồn bảo vệ chống cháy nổ.</t>
         </is>
       </c>
-      <c r="K8" s="3" t="n"/>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>[PASS] Động cơ hoạt động liên tục ổn định trong phòng kín nóng, không bị quá nhiệt.</t>
+        </is>
+      </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
           <t>Yes (Reviewed)</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -1008,10 +1071,19 @@
           <t>Thân quạt đứng vững, đế quạt bám chắc mặt sàn, độ rung lắc nằm trong biên độ nhỏ cho phép (&lt;5mm tại đỉnh lồng quạt).</t>
         </is>
       </c>
-      <c r="K9" s="5" t="n"/>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>[PASS] Đế quạt bám chắc và đứng vững vàng trên sàn phẳng.</t>
+        </is>
+      </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
           <t>Yes (Reviewed)</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1141,7 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>[FAIL] Khi quạt chạy tốc độ lớn nhất và xoay tu năng, lực rung động cơ và mô-men xoắn ly tâm làm quạt mất trọng tâm, lắc lư mạnh rồi đổ ngã khỏi bục gỗ cao 10cm.</t>
+          <t>[FAIL] Khi quạt chạy tốc độ lớn nhất và xoay tu năng, lực rung cơ học và lực ly tâm làm quạt mất trọng tâm và đổ ngã khỏi vật cao 10cm.</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1266,10 +1338,19 @@
           <t>Cơ cấu tu năng cơ học hoạt động nhạy, bắt khớp và nhả khớp bánh răng mượt mà, không bị kẹt hay trượt răng khi đổi trạng thái đột ngột.</t>
         </is>
       </c>
-      <c r="K13" s="5" t="n"/>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>[FAIL] Hoạt động không ổn định. Khi thực hiện giật/nhả tu năng và úp mở (ngẩng/cúi) liên tục thì cánh quạt có thể va chạm với lồng bảo vệ dẫn đến nguy hiểm cho người dùng.</t>
+        </is>
+      </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
           <t>Yes (Reviewed)</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
     </row>
@@ -1323,10 +1404,19 @@
           <t>Lồng quạt kim loại chắc chắn, không bị biến dạng dễ dàng, khoảng cách an toàn giữa lồng quạt và cánh quạt được duy trì tốt (khoảng cách &gt;1.5cm).</t>
         </is>
       </c>
-      <c r="K14" s="3" t="n"/>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>[PASS] Lồng quạt thép sơn tĩnh điện chịu lực tốt, không biến dạng chạm cánh.</t>
+        </is>
+      </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
           <t>Yes (Reviewed)</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -1380,10 +1470,19 @@
           <t>Khớp cổ quạt di chuyển nấc cơ học chắc chắn. Khi quạt chạy tốc độ 3, đầu quạt giữ nguyên góc điều chỉnh mà không bị xê dịch tự do dưới lực đẩy của gió.</t>
         </is>
       </c>
-      <c r="K15" s="5" t="n"/>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>[PASS] Đầu quạt định vị góc ngẩng/cúi chắc chắn, không bị xê dịch tự do khi chạy tốc độ cao.</t>
+        </is>
+      </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
           <t>Yes (Reviewed)</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
@@ -1437,10 +1536,19 @@
           <t>Độ ồn ở mức 1 phải đạt chuẩn Silent/Sleep (&lt;38dB), mức 2 &lt;45dB và mức 3 &lt;52dB.</t>
         </is>
       </c>
-      <c r="K16" s="3" t="n"/>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>[PASS] Độ ồn đo được ở khoảng cách 1m lần lượt là: 36dB (Silent), 43dB, 49dB (đạt tiêu chuẩn kỹ thuật thiết kế).</t>
+        </is>
+      </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
           <t>Yes (Reviewed)</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>

</xml_diff>